<commit_message>
Adicionado esqueleto de diretorios do projeto Caixa
</commit_message>
<xml_diff>
--- a/Projeto_1/data/Episodios_Simpsons.xlsx
+++ b/Projeto_1/data/Episodios_Simpsons.xlsx
@@ -2268,17 +2268,17 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "Adicionado esqueleto de diretorios do projeto Caixa"
This reverts commit 289821d41ca71b7d28a071ec386c05fc9f927c57.
</commit_message>
<xml_diff>
--- a/Projeto_1/data/Episodios_Simpsons.xlsx
+++ b/Projeto_1/data/Episodios_Simpsons.xlsx
@@ -2268,17 +2268,17 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TBA</t>
         </is>
       </c>
     </row>

</xml_diff>